<commit_message>
迁移 Campaign/Dashboard/AIManage/AdExtension/Adgroup 到 us/ 环境目录，合并 config 变量
- 按团队新目录规范把本session生成的5个模块搬到 single-api/mainapi/us/ 下
- us/config.json 补充 test_keyword_tag_id/adgroup_tag_id/adgroup_tag_owner_user_id/compare_start_mdy/compare_end_mdy
- update_excel.py 的 EXCEL_PATH 改回相对路径（Windows硬编码路径在mac上跑不了）
- 提交 single-api/run-cases.py（mac/python版执行引擎），修复 extract_vars 未实现、GET方法/query string不支持等问题
- 合并后重新对Campaign/Dashboard/AIManage/Adgroup跑了一遍Excel回填，落在同事最新的swagger_modules.xlsx上

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/single-api/swagger_modules.xlsx
+++ b/single-api/swagger_modules.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块汇总" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amazon.Advertising.Api" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PacvueMainApi" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="模块汇总" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Amazon.Advertising.Api" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="PacvueMainApi" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'模块汇总'!$A$1:$D$123</definedName>
@@ -910,6 +910,19 @@
           <t>guguangjie</t>
         </is>
       </c>
+      <c r="F6" s="29" t="n">
+        <v>31</v>
+      </c>
+      <c r="G6" s="29" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H6" s="29" t="inlineStr">
+        <is>
+          <t>100% (5/5)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="34" t="n"/>
@@ -986,6 +999,19 @@
           <t>guguangjie</t>
         </is>
       </c>
+      <c r="F9" s="29" t="n">
+        <v>101</v>
+      </c>
+      <c r="G9" s="29" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H9" s="29" t="inlineStr">
+        <is>
+          <t>100% (25/25)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="34" t="n"/>
@@ -1369,6 +1395,19 @@
           <t>guguangjie</t>
         </is>
       </c>
+      <c r="F24" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" s="29" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="H24" s="29" t="inlineStr">
+        <is>
+          <t>44% (4/9)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="34" t="n"/>
@@ -1519,6 +1558,19 @@
       <c r="E30" s="7" t="inlineStr">
         <is>
           <t>guguangjie</t>
+        </is>
+      </c>
+      <c r="F30" s="29" t="n">
+        <v>68</v>
+      </c>
+      <c r="G30" s="29" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="H30" s="29" t="inlineStr">
+        <is>
+          <t>90% (28/31)</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4366,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="96" customHeight="1">
       <c r="A22" s="34" t="n"/>
       <c r="B22" s="21" t="inlineStr">
         <is>
@@ -4336,8 +4388,18 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="23">
+      <c r="F22" s="37" t="inlineStr">
+        <is>
+          <t>单个Campaign详情页趋势图（按日Dim）
+按Campaign状态筛选的汇总趋势图（Dim=ytd）
+按状态+标签筛选的趋势图
+按名称搜索+状态筛选的趋势图
+无筛选查看全部Campaign整体趋势图
+按广告组合(Portfolio)+状态筛选的趋势图</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="80" customHeight="1">
       <c r="A23" s="34" t="n"/>
       <c r="B23" s="23" t="inlineStr">
         <is>
@@ -4359,8 +4421,17 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="24">
+      <c r="F23" s="37" t="inlineStr">
+        <is>
+          <t>按campaignId+campaignState+日期范围查询campaign列表
+按campaignId+日期范围查询campaign列表（不筛选状态）
+按campaignId+campaignName模糊搜索+campaignState+日期范围查询
+按campaignId+campaignState+广告类型(CampaignTypeItems)+日期范围查询
+按campaignId+campaignName模糊搜索+日期范围查询（不筛选状态）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="96" customHeight="1">
       <c r="A24" s="34" t="n"/>
       <c r="B24" s="22" t="inlineStr">
         <is>
@@ -4382,8 +4453,18 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="25">
+      <c r="F24" s="37" t="inlineStr">
+        <is>
+          <t>按指定CampaignId精确查询单个广告活动效果数据
+按状态筛选并附带同期对比查询广告活动列表
+按名称搜索并按状态筛选广告活动列表
+按状态和标签组合筛选广告活动列表
+无附加筛选条件的默认列表查询
+按广告类型(CampaignTypeItems)筛选广告活动列表</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="96" customHeight="1">
       <c r="A25" s="34" t="n"/>
       <c r="B25" s="23" t="inlineStr">
         <is>
@@ -4405,8 +4486,18 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="26">
+      <c r="F25" s="37" t="inlineStr">
+        <is>
+          <t>按效果指标筛选条件查询广告活动列表
+无筛选条件的默认活动列表查询
+按campaign标签(Tag)筛选查询
+按指定campaignIds批量精确查询
+按广告类型明细(CampaignTypeItems)筛选查询
+按广告组合(Portfolio)筛选查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="128" customHeight="1">
       <c r="A26" s="34" t="n"/>
       <c r="B26" s="22" t="inlineStr">
         <is>
@@ -4426,6 +4517,18 @@
       <c r="E26" s="7" t="inlineStr">
         <is>
           <t>guguangjie</t>
+        </is>
+      </c>
+      <c r="F26" s="37" t="inlineStr">
+        <is>
+          <t>场景1: 勾选指定Campaign汇总
+场景2: 按CampaignTag标签筛选汇总
+场景3: 按Campaign名称搜索汇总
+场景4: 默认总览 State筛选 同期对比
+场景5: 按投放状态ServingStatus筛选汇总
+场景6: 按Portfolio筛选汇总
+场景7: 按广告类型CampaignTypeItems筛选汇总
+场景8: 按目标Asin筛选汇总</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5131,7 @@
         </is>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="64" customHeight="1">
       <c r="A44" s="34" t="n"/>
       <c r="B44" s="21" t="inlineStr">
         <is>
@@ -5050,8 +5153,16 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="45">
+      <c r="F44" s="37" t="inlineStr">
+        <is>
+          <t>默认日粒度趋势查询(含环比对比期)
+按CampaignTag过滤的日粒度趋势查询
+周粒度(Dim=week)趋势查询
+月粒度(Dim=month)趋势查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="64" customHeight="1">
       <c r="A45" s="34" t="n"/>
       <c r="B45" s="23" t="inlineStr">
         <is>
@@ -5073,8 +5184,16 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="46">
+      <c r="F45" s="37" t="inlineStr">
+        <is>
+          <t>Brand+品类过滤日粒度Benchmark(无分享链接)
+不带Brand/品类过滤的整体Benchmark
+Brand+品类过滤且通过分享链接访问
+Brand+品类过滤且按周粒度(Dim=week)展示</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="48" customHeight="1">
       <c r="A46" s="34" t="n"/>
       <c r="B46" s="22" t="inlineStr">
         <is>
@@ -5096,8 +5215,15 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="47">
+      <c r="F46" s="37" t="inlineStr">
+        <is>
+          <t>单Profile按日期范围查询超预算广告活动列表
+多Profile跨店铺合并按日期范围查询超预算广告活动列表
+按Campaign Tag筛选查询超预算广告活动列表</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="48" customHeight="1">
       <c r="A47" s="34" t="n"/>
       <c r="B47" s="23" t="inlineStr">
         <is>
@@ -5119,8 +5245,15 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="48">
+      <c r="F47" s="37" t="inlineStr">
+        <is>
+          <t>基础日期范围查询Out of Budget图表（US市场，无标签/活动过滤）
+非US市场查询Out of Budget图表（汇率换算场景，以CA为代表）
+按CampaignTagId标签过滤的Out of Budget图表查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="80" customHeight="1">
       <c r="A48" s="34" t="n"/>
       <c r="B48" s="22" t="inlineStr">
         <is>
@@ -5142,8 +5275,17 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="49">
+      <c r="F48" s="37" t="inlineStr">
+        <is>
+          <t>US站点仅日期范围周对比周(单/多Profile聚合)
+非US市场(DE)基础周对比
+CampaignTagId标签过滤
+PortfolioId组合过滤
+ToMarket未指定(null)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="48" customHeight="1">
       <c r="A49" s="34" t="n"/>
       <c r="B49" s="23" t="inlineStr">
         <is>
@@ -5165,8 +5307,15 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="50">
+      <c r="F49" s="37" t="inlineStr">
+        <is>
+          <t>多账号Portfolio下钻子标签ROAS指标(滚动周期对比) — 45.5%
+单账号下钻子标签ROAS指标(月度环比) — 42.4%
+ACOS指标视角下钻子标签(年度累计vs去年同期对比) — 12.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="48" customHeight="1">
       <c r="A50" s="34" t="n"/>
       <c r="B50" s="22" t="inlineStr">
         <is>
@@ -5188,8 +5337,15 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="51">
+      <c r="F50" s="37" t="inlineStr">
+        <is>
+          <t>仅日期范围过滤查询Campaign Tag绩效widget(无Tag/Portfolio子筛选)
+按CampaignTagId筛选查询Campaign Tag绩效widget
+按PortfolioId筛选查询Campaign Tag绩效widget</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="48" customHeight="1">
       <c r="A51" s="34" t="n"/>
       <c r="B51" s="23" t="inlineStr">
         <is>
@@ -5211,8 +5367,15 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="52">
+      <c r="F51" s="37" t="inlineStr">
+        <is>
+          <t>查看标签ROAS目标达成率排名(默认汇率换算)
+查看标签ACOS目标达成率排名(默认汇率换算)
+查看标签ACOS目标达成率排名(不做汇率换算)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="80" customHeight="1">
       <c r="A52" s="34" t="n"/>
       <c r="B52" s="22" t="inlineStr">
         <is>
@@ -5234,8 +5397,17 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="53">
+      <c r="F52" s="37" t="inlineStr">
+        <is>
+          <t>场景1: 默认ROAS视图 无标签筛选 — 57.5%
+场景2: ACOS视图 新版CampaignTag命名 无筛选 — 14.2%
+场景3: ACOS视图 旧版Portfolio命名 无筛选 — 14.2%
+场景4: ACOS视图 按CampaignTagId筛选指定标签 — 8.4%
+场景5: ACOS视图 按旧版PortfolioId筛选 — 3.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="80" customHeight="1">
       <c r="A53" s="34" t="n"/>
       <c r="B53" s="23" t="inlineStr">
         <is>
@@ -5257,8 +5429,17 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="54">
+      <c r="F53" s="37" t="inlineStr">
+        <is>
+          <t>默认场景：仅日期范围过滤的 Top Performers（按 Spend 排序，开启汇率转换）
+未开启汇率转换（IsExchange=0）的 Top Performers 场景
+按 Campaign Tag 过滤的 Top Performers 场景
+按 Sales 排序对比且带自定义对比期的 Top Performers 场景
+Bottom Performers（performanceType=1）场景</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="48" customHeight="1">
       <c r="A54" s="34" t="n"/>
       <c r="B54" s="22" t="inlineStr">
         <is>
@@ -5280,8 +5461,15 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="55">
+      <c r="F54" s="37" t="inlineStr">
+        <is>
+          <t>仅按报表日期范围查询长尾词报表（无附加过滤）
+按广告系列标签(CampaignTagId)过滤查询长尾词报表
+按Amazon Portfolio(PortfolioId)过滤查询长尾词报表</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="80" customHeight="1">
       <c r="A55" s="34" t="n"/>
       <c r="B55" s="23" t="inlineStr">
         <is>
@@ -5303,8 +5491,17 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="56">
+      <c r="F55" s="37" t="inlineStr">
+        <is>
+          <t>单词(NumberOfWord=1)长尾关键词按MatchType报表(ROAS指标)
+双词(NumberOfWord=2)长尾关键词按MatchType报表
+三词(NumberOfWord=3)长尾关键词按MatchType报表
+四词(NumberOfWord=4)长尾关键词按MatchType报表
+分享报表(ShareId)+CampaignTagId标签过滤下的单词长尾关键词报表</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="64" customHeight="1">
       <c r="A56" s="34" t="n"/>
       <c r="B56" s="22" t="inlineStr">
         <is>
@@ -5326,8 +5523,16 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="57">
+      <c r="F56" s="37" t="inlineStr">
+        <is>
+          <t>基础场景:按天(Dim=date)+CampaignType(headlineSearch)筛选,无Tag/Portfolio筛选
+Campaign Tag筛选场景:附加CampaignTagId筛选,按天展示
+月粒度场景:Dim=month按月汇总展示
+Portfolio筛选场景:附加PortfolioId筛选,按天展示</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="64" customHeight="1">
       <c r="A57" s="34" t="n"/>
       <c r="B57" s="23" t="inlineStr">
         <is>
@@ -5349,8 +5554,16 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="58">
+      <c r="F57" s="37" t="inlineStr">
+        <is>
+          <t>单日期范围查询campaign类型层级绩效(无对比期无筛选)
+按日期范围并指定对比期查询campaign类型层级绩效
+按CampaignTagId筛选查询campaign类型层级绩效
+按PortfolioId筛选并指定对比期查询campaign类型层级绩效</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="96" customHeight="1">
       <c r="A58" s="34" t="n"/>
       <c r="B58" s="22" t="inlineStr">
         <is>
@@ -5372,8 +5585,18 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="59">
+      <c r="F58" s="37" t="inlineStr">
+        <is>
+          <t>Sponsored Products(SP)明细,单一日期范围(无对比期),ROAS指标
+Sponsored Brands(SB)明细,单一日期范围(无对比期),ROAS指标
+Sponsored Products(SP)明细,含对比期(环比/同比)
+Sponsored Brands(SB)明细,含对比期(环比/同比)
+按CampaignTagId(广告系列标签)筛选的明细查询
+按PortfolioId(广告组合)筛选的明细查询(含对比期)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="64" customHeight="1">
       <c r="A59" s="34" t="n"/>
       <c r="B59" s="23" t="inlineStr">
         <is>
@@ -5395,8 +5618,16 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="60">
+      <c r="F59" s="37" t="inlineStr">
+        <is>
+          <t>查询不合规商品(INELIGIBLE)明细列表
+查询缺货商品(NOT BUYABLE)明细列表
+查询未获得购物车商品(NOT IN BUYBOX)明细列表
+按CampaignTag筛选查询不合规商品(INELIGIBLE)明细列表</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="80" customHeight="1">
       <c r="A60" s="34" t="n"/>
       <c r="B60" s="22" t="inlineStr">
         <is>
@@ -5418,8 +5649,17 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="61">
+      <c r="F60" s="37" t="inlineStr">
+        <is>
+          <t>Top Search Terms 按 ROAS 排序（无额外筛选）
+Top Search Terms 按 ACOS 排序（无额外筛选）
+按 Campaign Tag 筛选查询 Top Search Terms
+按 Portfolio 筛选查询 Top Search Terms
+Poor Search Terms 查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="96" customHeight="1">
       <c r="A61" s="34" t="n"/>
       <c r="B61" s="23" t="inlineStr">
         <is>
@@ -5441,8 +5681,18 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="62">
+      <c r="F61" s="37" t="inlineStr">
+        <is>
+          <t>默认查询(无对比期,ROAS指标)
+带环比对比期查询(ROAS指标)
+默认查询(无对比期,ACOS指标)
+带对比期查询(ACOS指标,非US市场)
+按Campaign标签筛选查询
+按广告组合(Portfolio)筛选查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="64" customHeight="1">
       <c r="A62" s="34" t="n"/>
       <c r="B62" s="22" t="inlineStr">
         <is>
@@ -5464,8 +5714,16 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="63">
+      <c r="F62" s="37" t="inlineStr">
+        <is>
+          <t>多Profile(2-4个)组合非分享链路查询
+单Profile非分享链路查询
+多Profile组合通过分享链接(ShareId)访问
+大批量Profile(5个以上/近全选)组合查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="48" customHeight="1">
       <c r="A63" s="34" t="n"/>
       <c r="B63" s="23" t="inlineStr">
         <is>
@@ -5487,8 +5745,15 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="64">
+      <c r="F63" s="37" t="inlineStr">
+        <is>
+          <t>仅日期范围过滤查询周维度Campaign表现
+按CampaignTagId过滤查询周维度Campaign表现
+按PortfolioId过滤查询周维度Campaign表现</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="64" customHeight="1">
       <c r="A64" s="34" t="n"/>
       <c r="B64" s="22" t="inlineStr">
         <is>
@@ -5510,8 +5775,16 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="65">
+      <c r="F64" s="37" t="inlineStr">
+        <is>
+          <t>默认视图(ROAS指标,仅日期筛选,全部广告类型) — 73.6%
+ACOS指标视图(仅日期筛选,全部广告类型) — 17.2%
+按CampaignTag筛选(标签分组查看Placement绩效) — 5.4%
+按指定广告类型筛选(campaignType=1,非全部类型)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="48" customHeight="1">
       <c r="A65" s="34" t="n"/>
       <c r="B65" s="23" t="inlineStr">
         <is>
@@ -5533,8 +5806,15 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="66">
+      <c r="F65" s="37" t="inlineStr">
+        <is>
+          <t>按日期范围查询商品异常状态计数（无附加过滤）
+按广告系列标签(CampaignTagId)过滤后统计商品异常状态计数
+按广告组合(PortfolioId)过滤后统计商品异常状态计数</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="80" customHeight="1">
       <c r="A66" s="34" t="n"/>
       <c r="B66" s="22" t="inlineStr">
         <is>
@@ -5556,8 +5836,17 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="67">
+      <c r="F66" s="37" t="inlineStr">
+        <is>
+          <t>默认日期范围查询(多Profile,US市场)
+非美国市场(DE)日期范围查询
+按广告活动标签(CampaignTagId)过滤
+分享链接场景+广告活动标签过滤
+按广告组合(PortfolioId)过滤</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="64" customHeight="1">
       <c r="A67" s="34" t="n"/>
       <c r="B67" s="23" t="inlineStr">
         <is>
@@ -5579,8 +5868,16 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="68">
+      <c r="F67" s="37" t="inlineStr">
+        <is>
+          <t>仅日期范围过滤查询（美国市场，主流程）
+非美国市场日期范围查询（跨市场场景）
+按广告活动标签（CampaignTagId）过滤查询
+按 Portfolio ID 过滤查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="48" customHeight="1">
       <c r="A68" s="34" t="n"/>
       <c r="B68" s="22" t="inlineStr">
         <is>
@@ -5600,6 +5897,13 @@
       <c r="E68" s="7" t="inlineStr">
         <is>
           <t>guguangjie</t>
+        </is>
+      </c>
+      <c r="F68" s="37" t="inlineStr">
+        <is>
+          <t>默认日期范围查询(无标签/组合筛选)
+按CampaignTag标签筛选查询
+按Portfolio筛选查询</t>
         </is>
       </c>
     </row>
@@ -7929,7 +8233,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="16" customHeight="1">
       <c r="A28" s="34" t="n"/>
       <c r="B28" s="27" t="inlineStr">
         <is>
@@ -7951,8 +8255,13 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="29">
+      <c r="F28" s="37" t="inlineStr">
+        <is>
+          <t>冒烟测试(dev环境样本,非真实客户场景)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1">
       <c r="A29" s="34" t="n"/>
       <c r="B29" s="23" t="inlineStr">
         <is>
@@ -7972,6 +8281,11 @@
       <c r="E29" s="7" t="inlineStr">
         <is>
           <t>guguangjie</t>
+        </is>
+      </c>
+      <c r="F29" s="37" t="inlineStr">
+        <is>
+          <t>冒烟测试(dev环境样本,非真实客户场景)</t>
         </is>
       </c>
     </row>
@@ -7998,7 +8312,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="16" customHeight="1">
       <c r="A31" s="34" t="n"/>
       <c r="B31" s="23" t="inlineStr">
         <is>
@@ -8018,6 +8332,11 @@
       <c r="E31" s="7" t="inlineStr">
         <is>
           <t>guguangjie</t>
+        </is>
+      </c>
+      <c r="F31" s="37" t="inlineStr">
+        <is>
+          <t>冒烟测试(dev环境样本,默认分页,非真实客户场景)</t>
         </is>
       </c>
     </row>
@@ -8044,7 +8363,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="16" customHeight="1">
       <c r="A33" s="34" t="n"/>
       <c r="B33" s="23" t="inlineStr">
         <is>
@@ -8064,6 +8383,11 @@
       <c r="E33" s="7" t="inlineStr">
         <is>
           <t>guguangjie</t>
+        </is>
+      </c>
+      <c r="F33" s="37" t="inlineStr">
+        <is>
+          <t>冒烟测试(dev环境样本,非真实客户场景)</t>
         </is>
       </c>
     </row>
@@ -9553,7 +9877,7 @@
         </is>
       </c>
     </row>
-    <row r="96">
+    <row r="96" ht="64" customHeight="1">
       <c r="A96" s="34" t="n"/>
       <c r="B96" s="26" t="inlineStr">
         <is>
@@ -9575,8 +9899,16 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="97">
+      <c r="F96" s="37" t="inlineStr">
+        <is>
+          <t>场景1: 单AdGroup ASIN定向新增 — 29.8%
+场景2: 单AdGroup 自定义SKU编号定向新增 — 20.0%
+场景3: 多AdGroup批量 ASIN定向新增 — 35.4%
+场景4: 多AdGroup批量 自定义SKU编号定向新增 — 14.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="48" customHeight="1">
       <c r="A97" s="34" t="n"/>
       <c r="B97" s="23" t="inlineStr">
         <is>
@@ -9598,8 +9930,15 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="98">
+      <c r="F97" s="37" t="inlineStr">
+        <is>
+          <t>场景1: 单个SP广告组少量ASIN添加(1-4个)
+场景2: SP广告组中等批量多规格SKU添加(5-49个)
+场景3: SP广告组大批量SKU导入(≥50个,整店同步)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="48" customHeight="1">
       <c r="A98" s="34" t="n"/>
       <c r="B98" s="27" t="inlineStr">
         <is>
@@ -9619,6 +9958,13 @@
       <c r="E98" s="7" t="inlineStr">
         <is>
           <t>guguangjie</t>
+        </is>
+      </c>
+      <c r="F98" s="37" t="inlineStr">
+        <is>
+          <t>单广告组添加单个ASIN商品定向(含后置归档,可重复) — 27%
+单广告组批量粘贴多个ASIN商品定向(含后置归档,可重复) — 33%
+跨多个广告组批量应用同一ASIN商品定向(含后置归档,可重复) — 40%</t>
         </is>
       </c>
     </row>
@@ -9668,7 +10014,7 @@
         </is>
       </c>
     </row>
-    <row r="101">
+    <row r="101" ht="48" customHeight="1">
       <c r="A101" s="34" t="n"/>
       <c r="B101" s="23" t="inlineStr">
         <is>
@@ -9690,8 +10036,15 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="102">
+      <c r="F101" s="37" t="inlineStr">
+        <is>
+          <t>Campaign级批量创建否定精确匹配关键词(SP)
+Campaign级批量创建否定词组匹配关键词(SB)
+AdGroup级批量创建否定关键词(SP手动/PAT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="32" customHeight="1">
       <c r="A102" s="34" t="n"/>
       <c r="B102" s="27" t="inlineStr">
         <is>
@@ -9713,8 +10066,14 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="103">
+      <c r="F102" s="37" t="inlineStr">
+        <is>
+          <t>SP广告组仅设置ROAS竞价优化目标(ACOS未设置/高频场景)
+SP手动/PAT广告组同时设置ACOS与ROAS双竞价优化目标(中频场景)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="48" customHeight="1">
       <c r="A103" s="34" t="n"/>
       <c r="B103" s="23" t="inlineStr">
         <is>
@@ -9734,6 +10093,13 @@
       <c r="E103" s="7" t="inlineStr">
         <is>
           <t>guguangjie</t>
+        </is>
+      </c>
+      <c r="F103" s="37" t="inlineStr">
+        <is>
+          <t>场景1: 单ASIN替换 旧目标转Paused 新目标默认 — 90.9%
+场景2: 全字段显式替换 旧目标Archived 新目标Enabled keep=false — 7.07%
+场景3: 保留旧目标keep=true 新增替换目标Paused — 2.02%</t>
         </is>
       </c>
     </row>
@@ -9852,7 +10218,7 @@
         </is>
       </c>
     </row>
-    <row r="109">
+    <row r="109" ht="48" customHeight="1">
       <c r="A109" s="34" t="n"/>
       <c r="B109" s="23" t="inlineStr">
         <is>
@@ -9874,8 +10240,15 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="110">
+      <c r="F109" s="37" t="inlineStr">
+        <is>
+          <t>CopyAdGroup SP Manual ToDifferentCampaign — 63.8%
+CopyAdGroup SP Manual SameCampaign Duplicate — 17.7%
+CopyAdGroup SP Auto ToDifferentCampaign — 15.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="48" customHeight="1">
       <c r="A110" s="34" t="n"/>
       <c r="B110" s="27" t="inlineStr">
         <is>
@@ -9895,6 +10268,13 @@
       <c r="E110" s="7" t="inlineStr">
         <is>
           <t>guguangjie</t>
+        </is>
+      </c>
+      <c r="F110" s="37" t="inlineStr">
+        <is>
+          <t>场景1: SP手动投放AdGroup单ASIN复制 — 82.4%
+场景2: SP自动投放AdGroup单ASIN复制 — 6.8%
+场景3: SP手动投放AdGroup多ASIN复制 — 8.1%</t>
         </is>
       </c>
     </row>
@@ -9921,7 +10301,7 @@
         </is>
       </c>
     </row>
-    <row r="112">
+    <row r="112" ht="16" customHeight="1">
       <c r="A112" s="34" t="n"/>
       <c r="B112" s="27" t="inlineStr">
         <is>
@@ -9943,8 +10323,13 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="113">
+      <c r="F112" s="37" t="inlineStr">
+        <is>
+          <t>复制SponsoredDisplay广告组（manual targeting，同campaign内复制）</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="16" customHeight="1">
       <c r="A113" s="34" t="n"/>
       <c r="B113" s="23" t="inlineStr">
         <is>
@@ -9964,6 +10349,11 @@
       <c r="E113" s="7" t="inlineStr">
         <is>
           <t>guguangjie</t>
+        </is>
+      </c>
+      <c r="F113" s="37" t="inlineStr">
+        <is>
+          <t>复制SD广告组(含创意+ASIN定向,含后置清理,可重复)</t>
         </is>
       </c>
     </row>
@@ -9990,7 +10380,7 @@
         </is>
       </c>
     </row>
-    <row r="115">
+    <row r="115" ht="304" customHeight="1">
       <c r="A115" s="34" t="n"/>
       <c r="B115" s="23" t="inlineStr">
         <is>
@@ -10012,8 +10402,31 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="116">
+      <c r="F115" s="37" t="inlineStr">
+        <is>
+          <t>SP单个AdGroup批量改价（高频场景）
+SP多个AdGroup跨Campaign批量改价（中频场景）
+跨广告类型批量改价含SD设置bidOptimization（中频场景）
+场景1: SponsoredProducts通用场景 启用AdGroup
+场景2: SponsoredProducts手动PAT场景 暂停AdGroup
+场景3: SponsoredDisplay场景 切换AdGroup状态
+场景4: SponsoredProducts通用场景 归档AdGroup
+批量设置SD广告组优化方式为clicks(前置读原值+后置还原,可重复)
+通过全局唯一id查询广告组编辑数据 — 60%
+通过profileId+campaignId+adGroupId组合查询广告组编辑数据 — 10%
+低价位默认出价调整(&lt;1,含读原值+还原) — 50.8%
+中价位默认出价调整(1~3,含读原值+还原) — 40.9%
+高价位默认出价调整(&gt;3,含读原值+还原) — 8.3%
+SD AdGroup Update Basic Attributes NoCostControl
+SD AdGroup Update EnableCostControl
+SD AdGroup Update DisableCostControl
+批量修改AdGroup名称(含读原值+还原,可重复)
+普通改名场景-读取原名后改名并还原
+带sourceName(Creative Hub来源)的改名场景-读取原名后改名并还原</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="48" customHeight="1">
       <c r="A116" s="34" t="n"/>
       <c r="B116" s="27" t="inlineStr">
         <is>
@@ -10033,6 +10446,13 @@
       <c r="E116" s="7" t="inlineStr">
         <is>
           <t>guguangjie</t>
+        </is>
+      </c>
+      <c r="F116" s="37" t="inlineStr">
+        <is>
+          <t>不指定CampaignIds查询全部候选AdGroup — 61.4%
+单个CampaignId查询PAT研究AdGroup — 36.8%
+多个CampaignIds批量查询PAT研究AdGroup — 1.8%</t>
         </is>
       </c>
     </row>
@@ -10059,7 +10479,7 @@
         </is>
       </c>
     </row>
-    <row r="118">
+    <row r="118" ht="80" customHeight="1">
       <c r="A118" s="34" t="n"/>
       <c r="B118" s="27" t="inlineStr">
         <is>
@@ -10081,8 +10501,17 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="119">
+      <c r="F118" s="37" t="inlineStr">
+        <is>
+          <t>SB广告活动详情页-单Campaign级Adgroup趋势图（按周Dim）
+Adgroup列表页-账户级总览趋势图（不筛选任何Campaign/AdGroup）
+AdGroup Tag聚合分析-跨Profile的Tag维度Adgroup趋势图
+Adgroup列表页-按Portfolio筛选后的趋势图
+Adgroup列表页-钻取到指定AdGroup的趋势图</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="64" customHeight="1">
       <c r="A119" s="34" t="n"/>
       <c r="B119" s="23" t="inlineStr">
         <is>
@@ -10104,8 +10533,16 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="120">
+      <c r="F119" s="37" t="inlineStr">
+        <is>
+          <t>按Campaign查看AdGroup列表(不限定具体AdGroup) — 43.6%
+AdGroup模块主列表(默认活跃状态,不限Campaign) — 25.8%
+AdGroup模块主列表(按AdGroup标签筛选) — 25.6%
+Campaign详情钻取查看单个AdGroup — 4.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="48" customHeight="1">
       <c r="A120" s="34" t="n"/>
       <c r="B120" s="27" t="inlineStr">
         <is>
@@ -10127,8 +10564,15 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="121">
+      <c r="F120" s="37" t="inlineStr">
+        <is>
+          <t>campaignId查询AdgroupTotal 单campaign汇总
+campaignId加adgroupId查询AdgroupTotal 指定adgroup汇总
+广告类型加状态过滤查询AdgroupTotal 账户级汇总</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="48" customHeight="1">
       <c r="A121" s="34" t="n"/>
       <c r="B121" s="23" t="inlineStr">
         <is>
@@ -10150,8 +10594,15 @@
           <t>guguangjie</t>
         </is>
       </c>
-    </row>
-    <row r="122">
+      <c r="F121" s="37" t="inlineStr">
+        <is>
+          <t>查询SP手动定位(PAT)广告系列的广告组类型
+查询SP通用广告系列的广告组类型
+查询SD广告系列的广告组类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="80" customHeight="1">
       <c r="A122" s="34" t="n"/>
       <c r="B122" s="27" t="inlineStr">
         <is>
@@ -10171,6 +10622,15 @@
       <c r="E122" s="7" t="inlineStr">
         <is>
           <t>guguangjie</t>
+        </is>
+      </c>
+      <c r="F122" s="37" t="inlineStr">
+        <is>
+          <t>场景1: 同Campaign内复制并保持enabled
+场景2: 同Campaign内复制并保持paused
+单个SP广告系列查询广告组列表 — 92.7%
+单个SD广告系列查询广告组列表 — 92.7%
+批量多campaignId查询广告组列表 — 7.3%</t>
         </is>
       </c>
     </row>

</xml_diff>